<commit_message>
Add carousel-training block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (15):
- blocks/carousel-training/carousel-training.css
- blocks/carousel-training/carousel-training.js
- package-lock.json
- package.json
- tools/importer/import-roles-finder.bundle.js
- tools/importer/import-roles-finder.js
- tools/importer/page-templates.json
- tools/importer/parsers/carousel-training.js
- tools/importer/parsers/columns-dualpanel.js
- tools/importer/reports/import-roles-finder.report.xlsx
- tools/importer/reports/roles/roles-finder/aircrew/pilot.report.json
- tools/importer/reports/roles/roles-finder/aircrew/weapon-systems-officer.report.json
- tools/importer/reports/roles/roles-finder/aircrew/weapon-systems-operator-aircrew-linguist.report.json
- tools/importer/reports/roles/roles-finder/aircrew/weapon-systems-operator.report.json
- tools/importer/transformers/raf-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-roles-finder.report.xlsx
+++ b/tools/importer/reports/import-roles-finder.report.xlsx
@@ -40,7 +40,7 @@
     <t>roles/roles-finder/aircrew/pilot.report.json</t>
   </si>
   <si>
-    <t>["hero","hero","hero","columns-roleinfo","columns","accordion","carousel-training","section-whyjoin-officer","section-whyjoin-officer","cards-benefits","carousel-steps","columns-cta","cards-roles","section-contact","section-contact"]</t>
+    <t>["hero","hero","hero","columns-roleinfo","columns","accordion","carousel-training","section-whyjoin-officer","section-whyjoin-officer","cards-benefits","carousel-steps","columns-cta","cards-roles","section-contact"]</t>
   </si>
   <si>
     <t>roles/roles-finder/aircrew/pilot</t>
@@ -52,7 +52,7 @@
     <t>roles-finder</t>
   </si>
   <si>
-    <t>2026-03-06T22:34:09.956Z</t>
+    <t>2026-03-10T22:56:48.138Z</t>
   </si>
   <si>
     <t>RAF Recruitment | Pilot | Royal Air Force</t>
@@ -64,13 +64,13 @@
     <t>roles/roles-finder/aircrew/weapon-systems-officer.report.json</t>
   </si>
   <si>
-    <t>["hero","hero","hero","columns-roleinfo","columns","columns","accordion","carousel-training","section-whyjoin-officer","cards-benefits","carousel-steps","columns-cta","cards-roles","section-contact","section-contact"]</t>
+    <t>["hero","hero","hero","columns-roleinfo","columns","accordion","carousel-training","section-whyjoin-officer","cards-benefits","carousel-steps","columns-cta","cards-roles","section-contact"]</t>
   </si>
   <si>
     <t>roles/roles-finder/aircrew/weapon-systems-officer</t>
   </si>
   <si>
-    <t>2026-03-06T22:33:19.731Z</t>
+    <t>2026-03-10T22:56:00.795Z</t>
   </si>
   <si>
     <t>RAF Recruitment | Weapon Systems Officer | Royal Air Force</t>
@@ -82,13 +82,13 @@
     <t>roles/roles-finder/aircrew/weapon-systems-operator-aircrew-linguist.report.json</t>
   </si>
   <si>
-    <t>["hero","hero","hero","columns-roleinfo","columns","columns","accordion","carousel-training","cards-benefits","carousel-steps","columns-cta","cards-roles","section-contact","section-contact"]</t>
+    <t>["hero","hero","hero","columns-roleinfo","columns","accordion","carousel-training","cards-benefits","carousel-steps","columns-cta","cards-roles","section-contact"]</t>
   </si>
   <si>
     <t>roles/roles-finder/aircrew/weapon-systems-operator-aircrew-linguist</t>
   </si>
   <si>
-    <t>2026-03-06T22:33:50.598Z</t>
+    <t>2026-03-10T22:56:33.387Z</t>
   </si>
   <si>
     <t>RAF Recruitment | Weapon Systems Operator - Aircrew Linguist | Royal Air Force</t>
@@ -103,7 +103,7 @@
     <t>roles/roles-finder/aircrew/weapon-systems-operator</t>
   </si>
   <si>
-    <t>2026-03-06T22:33:34.403Z</t>
+    <t>2026-03-10T22:56:16.409Z</t>
   </si>
   <si>
     <t>RAF Recruitment | Weapon Systems Operator | Royal Air Force</t>

</xml_diff>